<commit_message>
add new_account and upgrade_castle method for Castle.
</commit_message>
<xml_diff>
--- a/data/WAO_farms_data.xlsx
+++ b/data/WAO_farms_data.xlsx
@@ -2,34 +2,51 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Arial"/>
+      <charset val="1"/>
+      <family val="2"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <scheme val="minor"/>
+      <family val="0"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color theme="1"/>
-      <scheme val="minor"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,29 +54,56 @@
       <patternFill/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom"/>
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -133,9 +177,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -143,127 +187,105 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="EEECE1"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="1F497D"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285F4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="EA4335"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="FBBC04"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34A853"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="FF6D01"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46BDC6"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="SimSun" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Times New Roman" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -274,51 +296,54 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -328,237 +353,249 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Z8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:Z9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col width="14" customWidth="1" style="5" min="6" max="6"/>
+    <col width="14" customWidth="1" style="3" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="4">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>lv</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>google</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>account</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>alliance</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>marches_limit</t>
         </is>
       </c>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
-      <c r="I1" s="3" t="n"/>
-      <c r="J1" s="3" t="n"/>
-      <c r="K1" s="3" t="n"/>
-      <c r="L1" s="3" t="n"/>
-      <c r="M1" s="3" t="n"/>
-      <c r="N1" s="3" t="n"/>
-      <c r="O1" s="3" t="n"/>
-      <c r="P1" s="3" t="n"/>
-      <c r="Q1" s="3" t="n"/>
-      <c r="R1" s="3" t="n"/>
-      <c r="S1" s="3" t="n"/>
-      <c r="T1" s="3" t="n"/>
-      <c r="U1" s="3" t="n"/>
-      <c r="V1" s="3" t="n"/>
-      <c r="W1" s="3" t="n"/>
-      <c r="X1" s="3" t="n"/>
-      <c r="Y1" s="3" t="n"/>
-      <c r="Z1" s="3" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="G1" s="6" t="n"/>
+      <c r="H1" s="6" t="n"/>
+      <c r="I1" s="6" t="n"/>
+      <c r="J1" s="6" t="n"/>
+      <c r="K1" s="6" t="n"/>
+      <c r="L1" s="6" t="n"/>
+      <c r="M1" s="6" t="n"/>
+      <c r="N1" s="6" t="n"/>
+      <c r="O1" s="6" t="n"/>
+      <c r="P1" s="6" t="n"/>
+      <c r="Q1" s="6" t="n"/>
+      <c r="R1" s="6" t="n"/>
+      <c r="S1" s="6" t="n"/>
+      <c r="T1" s="6" t="n"/>
+      <c r="U1" s="6" t="n"/>
+      <c r="V1" s="6" t="n"/>
+      <c r="W1" s="6" t="n"/>
+      <c r="X1" s="6" t="n"/>
+      <c r="Y1" s="6" t="n"/>
+      <c r="Z1" s="6" t="n"/>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="4">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>leo</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>
       </c>
-      <c r="F2" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="F2" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" s="4">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>haac</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>MIA</t>
         </is>
       </c>
-      <c r="F3" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="F3" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1" s="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>hac</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>MIA</t>
         </is>
       </c>
-      <c r="F4" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="F4" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" s="4">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>farm,hacen</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>ViC</t>
         </is>
       </c>
-      <c r="F5" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="F5" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" s="4">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>VIChac</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>MIA</t>
         </is>
       </c>
-      <c r="F6" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="F6" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" s="4">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>kazuru_farm5</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="4" t="n">
+      <c r="C7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>MIA</t>
         </is>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="3" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="8" ht="15.75" customHeight="1" s="4">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>kazuru_farm6</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="C8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>MIA</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="3" t="n">
         <v>2</v>
       </c>
     </row>
+    <row r="9" ht="15.75" customHeight="1" s="4">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="overThenDown" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
• fix new_account and close_ad stability across inconsistent UI states      • add claim_rss, claim_quest, and events routines to broaden daily automation coverage      • improve heal, to_map, and account status handling for fresh accounts      • add speed_up, research, forge, and kill_monster flows with safer retries and fallbacks      • introduce log_raise helper for clearer, actionable failures when critical steps cannot proceed
</commit_message>
<xml_diff>
--- a/data/WAO_farms_data.xlsx
+++ b/data/WAO_farms_data.xlsx
@@ -76,7 +76,10 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -360,237 +363,240 @@
   <dimension ref="A1:Z9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col width="14" customWidth="1" style="3" min="6" max="6"/>
+    <col width="14" customWidth="1" style="4" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="4">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="5">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>lv</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>google</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>account</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>alliance</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>marches_limit</t>
         </is>
       </c>
-      <c r="G1" s="6" t="n"/>
-      <c r="H1" s="6" t="n"/>
-      <c r="I1" s="6" t="n"/>
-      <c r="J1" s="6" t="n"/>
-      <c r="K1" s="6" t="n"/>
-      <c r="L1" s="6" t="n"/>
-      <c r="M1" s="6" t="n"/>
-      <c r="N1" s="6" t="n"/>
-      <c r="O1" s="6" t="n"/>
-      <c r="P1" s="6" t="n"/>
-      <c r="Q1" s="6" t="n"/>
-      <c r="R1" s="6" t="n"/>
-      <c r="S1" s="6" t="n"/>
-      <c r="T1" s="6" t="n"/>
-      <c r="U1" s="6" t="n"/>
-      <c r="V1" s="6" t="n"/>
-      <c r="W1" s="6" t="n"/>
-      <c r="X1" s="6" t="n"/>
-      <c r="Y1" s="6" t="n"/>
-      <c r="Z1" s="6" t="n"/>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" s="4">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="7" t="n"/>
+      <c r="I1" s="7" t="n"/>
+      <c r="J1" s="7" t="n"/>
+      <c r="K1" s="7" t="n"/>
+      <c r="L1" s="7" t="n"/>
+      <c r="M1" s="7" t="n"/>
+      <c r="N1" s="7" t="n"/>
+      <c r="O1" s="7" t="n"/>
+      <c r="P1" s="7" t="n"/>
+      <c r="Q1" s="7" t="n"/>
+      <c r="R1" s="7" t="n"/>
+      <c r="S1" s="7" t="n"/>
+      <c r="T1" s="7" t="n"/>
+      <c r="U1" s="7" t="n"/>
+      <c r="V1" s="7" t="n"/>
+      <c r="W1" s="7" t="n"/>
+      <c r="X1" s="7" t="n"/>
+      <c r="Y1" s="7" t="n"/>
+      <c r="Z1" s="7" t="n"/>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="5">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>VIChac</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" s="5">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>farm,hacen</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>ViC</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1" s="5">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>leo</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F4" s="4" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" s="4">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="5" ht="15.75" customHeight="1" s="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>kazuru_farm6</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" s="5">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>kazuru_farm5</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" s="5">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>hac</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1" s="5">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>haac</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B8" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>MIA</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F8" s="4" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" s="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>hac</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C4" s="3" t="n">
+    <row r="9" ht="15.75" customHeight="1" s="5">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" s="4">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>farm,hacen</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>ViC</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" s="4">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>VIChac</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" s="4">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>kazuru_farm5</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" s="4">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>kazuru_farm6</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" s="4">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>